<commit_message>
Sumo nuevas estimaciones lapop
</commit_message>
<xml_diff>
--- a/Output/municipal_pre_controls_all_pre_years.xlsx
+++ b/Output/municipal_pre_controls_all_pre_years.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t xml:space="preserve">mun_code</t>
   </si>
@@ -38,19 +38,16 @@
     <t xml:space="preserve">mun_pre_all_share_en_pareja</t>
   </si>
   <si>
-    <t xml:space="preserve">mun_pre_all_share_etnia_minoritaria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mun_pre_all_share_secundaria_completa_o_mas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mun_pre_all_share_superior_incompleta_o_mas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mun_pre_all_share_superior_completa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mun_pre_all_share_blanco</t>
+    <t xml:space="preserve">mun_pre_all_mean_educ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mun_pre_all_mean_izq_der</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mun_pre_all_share_interes_pol_mucho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mun_pre_all_share_voto_blanco_nulo</t>
   </si>
   <si>
     <t xml:space="preserve">002001</t>
@@ -578,13 +575,10 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2" t="n">
         <v>42.5637450199203</v>
@@ -608,22 +602,21 @@
         <v>0.486111111111111</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0334728033472803</v>
+        <v>11.8796498905908</v>
       </c>
       <c r="J2" t="n">
-        <v>0.663019693654267</v>
+        <v>5.07692307692308</v>
       </c>
       <c r="K2" t="n">
-        <v>0.389496717724289</v>
+        <v>0.218436873747495</v>
       </c>
       <c r="L2" t="n">
-        <v>0.12691466083151</v>
-      </c>
-      <c r="M2"/>
+        <v>0.0997304582210243</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" t="n">
         <v>43.375</v>
@@ -647,22 +640,21 @@
         <v>0.616438356164384</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0277777777777778</v>
+        <v>11.5230769230769</v>
       </c>
       <c r="J3" t="n">
-        <v>0.584615384615385</v>
+        <v>5.56896551724138</v>
       </c>
       <c r="K3" t="n">
-        <v>0.384615384615385</v>
+        <v>0.23943661971831</v>
       </c>
       <c r="L3" t="n">
-        <v>0.153846153846154</v>
-      </c>
-      <c r="M3"/>
+        <v>0.0967741935483871</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" t="n">
         <v>42.1780821917808</v>
@@ -686,22 +678,21 @@
         <v>0.468965517241379</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0220588235294118</v>
+        <v>11.0071428571429</v>
       </c>
       <c r="J4" t="n">
-        <v>0.585714285714286</v>
+        <v>4.828125</v>
       </c>
       <c r="K4" t="n">
-        <v>0.4</v>
+        <v>0.157534246575342</v>
       </c>
       <c r="L4" t="n">
-        <v>0.107142857142857</v>
-      </c>
-      <c r="M4"/>
+        <v>0.0983606557377049</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B5" t="n">
         <v>41.625</v>
@@ -725,22 +716,21 @@
         <v>0.583333333333333</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0140845070422535</v>
+        <v>11.1142857142857</v>
       </c>
       <c r="J5" t="n">
-        <v>0.585714285714286</v>
+        <v>5.3968253968254</v>
       </c>
       <c r="K5" t="n">
-        <v>0.342857142857143</v>
+        <v>0.0833333333333333</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0857142857142857</v>
-      </c>
-      <c r="M5"/>
+        <v>0.125</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" t="n">
         <v>42.5694444444444</v>
@@ -764,22 +754,21 @@
         <v>0.638888888888889</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0606060606060606</v>
+        <v>10.6760563380282</v>
       </c>
       <c r="J6" t="n">
-        <v>0.47887323943662</v>
+        <v>5.05357142857143</v>
       </c>
       <c r="K6" t="n">
-        <v>0.225352112676056</v>
+        <v>0.111111111111111</v>
       </c>
       <c r="L6" t="n">
-        <v>0.0563380281690141</v>
-      </c>
-      <c r="M6"/>
+        <v>0.2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" t="n">
         <v>41.6805555555556</v>
@@ -803,22 +792,21 @@
         <v>0.576388888888889</v>
       </c>
       <c r="I7" t="n">
-        <v>0.046875</v>
+        <v>9.47552447552447</v>
       </c>
       <c r="J7" t="n">
-        <v>0.307692307692308</v>
+        <v>5.4622641509434</v>
       </c>
       <c r="K7" t="n">
-        <v>0.167832167832168</v>
+        <v>0.119718309859155</v>
       </c>
       <c r="L7" t="n">
-        <v>0.048951048951049</v>
-      </c>
-      <c r="M7"/>
+        <v>0.135922330097087</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B8" t="n">
         <v>40.75</v>
@@ -842,22 +830,21 @@
         <v>0.555555555555556</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0714285714285714</v>
+        <v>9.97183098591549</v>
       </c>
       <c r="J8" t="n">
-        <v>0.408450704225352</v>
+        <v>5.67796610169492</v>
       </c>
       <c r="K8" t="n">
-        <v>0.211267605633803</v>
+        <v>0.0833333333333333</v>
       </c>
       <c r="L8" t="n">
-        <v>0.0422535211267606</v>
-      </c>
-      <c r="M8"/>
+        <v>0.163934426229508</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B9" t="n">
         <v>41.027397260274</v>
@@ -881,22 +868,21 @@
         <v>0.684931506849315</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0294117647058824</v>
+        <v>9.34246575342466</v>
       </c>
       <c r="J9" t="n">
-        <v>0.36986301369863</v>
+        <v>5.42424242424242</v>
       </c>
       <c r="K9" t="n">
-        <v>0.136986301369863</v>
+        <v>0.0821917808219178</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0410958904109589</v>
-      </c>
-      <c r="M9"/>
+        <v>0.133333333333333</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10" t="n">
         <v>43</v>
@@ -920,22 +906,21 @@
         <v>0.444444444444444</v>
       </c>
       <c r="I10" t="n">
-        <v>0.0307692307692308</v>
+        <v>10.3478260869565</v>
       </c>
       <c r="J10" t="n">
-        <v>0.478260869565217</v>
+        <v>5.33333333333333</v>
       </c>
       <c r="K10" t="n">
-        <v>0.260869565217391</v>
+        <v>0.185714285714286</v>
       </c>
       <c r="L10" t="n">
-        <v>0.0289855072463768</v>
-      </c>
-      <c r="M10"/>
+        <v>0.163636363636364</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B11" t="n">
         <v>42.9861111111111</v>
@@ -959,22 +944,21 @@
         <v>0.534246575342466</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0169491525423729</v>
+        <v>10.8142857142857</v>
       </c>
       <c r="J11" t="n">
-        <v>0.557142857142857</v>
+        <v>5.28333333333333</v>
       </c>
       <c r="K11" t="n">
-        <v>0.342857142857143</v>
+        <v>0.0821917808219178</v>
       </c>
       <c r="L11" t="n">
-        <v>0.0571428571428571</v>
-      </c>
-      <c r="M11"/>
+        <v>0.109375</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B12" t="n">
         <v>41.625</v>
@@ -998,22 +982,21 @@
         <v>0.527777777777778</v>
       </c>
       <c r="I12" t="n">
-        <v>0.0149253731343284</v>
+        <v>9.18571428571429</v>
       </c>
       <c r="J12" t="n">
-        <v>0.357142857142857</v>
+        <v>5.0377358490566</v>
       </c>
       <c r="K12" t="n">
-        <v>0.0857142857142857</v>
+        <v>0.1</v>
       </c>
       <c r="L12" t="n">
-        <v>0.0285714285714286</v>
-      </c>
-      <c r="M12"/>
+        <v>0.218181818181818</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B13" t="n">
         <v>43.6805555555556</v>
@@ -1037,22 +1020,21 @@
         <v>0.527777777777778</v>
       </c>
       <c r="I13" t="n">
-        <v>0.0461538461538462</v>
+        <v>9.19444444444444</v>
       </c>
       <c r="J13" t="n">
-        <v>0.375</v>
+        <v>5.73584905660377</v>
       </c>
       <c r="K13" t="n">
-        <v>0.152777777777778</v>
+        <v>0.138888888888889</v>
       </c>
       <c r="L13" t="n">
-        <v>0.0277777777777778</v>
-      </c>
-      <c r="M13"/>
+        <v>0.103448275862069</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B14" t="n">
         <v>43.2638888888889</v>
@@ -1076,22 +1058,21 @@
         <v>0.486111111111111</v>
       </c>
       <c r="I14" t="n">
-        <v>0.0149253731343284</v>
+        <v>9.33802816901408</v>
       </c>
       <c r="J14" t="n">
-        <v>0.394366197183099</v>
+        <v>5.59649122807018</v>
       </c>
       <c r="K14" t="n">
-        <v>0.197183098591549</v>
+        <v>0.222222222222222</v>
       </c>
       <c r="L14" t="n">
-        <v>0.0563380281690141</v>
-      </c>
-      <c r="M14"/>
+        <v>0.180327868852459</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B15" t="n">
         <v>41.5264623955432</v>
@@ -1115,22 +1096,21 @@
         <v>0.545706371191136</v>
       </c>
       <c r="I15" t="n">
-        <v>0.0578778135048231</v>
+        <v>9.56179775280899</v>
       </c>
       <c r="J15" t="n">
-        <v>0.370786516853933</v>
+        <v>5.49828178694158</v>
       </c>
       <c r="K15" t="n">
-        <v>0.199438202247191</v>
+        <v>0.143258426966292</v>
       </c>
       <c r="L15" t="n">
-        <v>0.0252808988764045</v>
-      </c>
-      <c r="M15"/>
+        <v>0.145593869731801</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B16" t="n">
         <v>43.6301369863014</v>
@@ -1154,22 +1134,21 @@
         <v>0.486111111111111</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>12.4029850746269</v>
       </c>
       <c r="J16" t="n">
-        <v>0.776119402985075</v>
+        <v>5.16666666666667</v>
       </c>
       <c r="K16" t="n">
-        <v>0.447761194029851</v>
+        <v>0.263888888888889</v>
       </c>
       <c r="L16" t="n">
-        <v>0.119402985074627</v>
-      </c>
-      <c r="M16"/>
+        <v>0.0961538461538462</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B17" t="n">
         <v>43.6666666666667</v>
@@ -1193,22 +1172,21 @@
         <v>0.597222222222222</v>
       </c>
       <c r="I17" t="n">
-        <v>0.0317460317460317</v>
+        <v>11.5588235294118</v>
       </c>
       <c r="J17" t="n">
-        <v>0.558823529411765</v>
+        <v>5.06349206349206</v>
       </c>
       <c r="K17" t="n">
-        <v>0.352941176470588</v>
+        <v>0.23943661971831</v>
       </c>
       <c r="L17" t="n">
-        <v>0.0882352941176471</v>
-      </c>
-      <c r="M17"/>
+        <v>0.135593220338983</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B18" t="n">
         <v>42.2602739726027</v>
@@ -1232,22 +1210,21 @@
         <v>0.602739726027397</v>
       </c>
       <c r="I18" t="n">
-        <v>0.028169014084507</v>
+        <v>11.0857142857143</v>
       </c>
       <c r="J18" t="n">
-        <v>0.514285714285714</v>
+        <v>5.03030303030303</v>
       </c>
       <c r="K18" t="n">
-        <v>0.371428571428571</v>
+        <v>0.125</v>
       </c>
       <c r="L18" t="n">
-        <v>0.114285714285714</v>
-      </c>
-      <c r="M18"/>
+        <v>0.109090909090909</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B19" t="n">
         <v>41.3287671232877</v>
@@ -1271,22 +1248,21 @@
         <v>0.602739726027397</v>
       </c>
       <c r="I19" t="n">
-        <v>0.0454545454545455</v>
+        <v>11.8028169014085</v>
       </c>
       <c r="J19" t="n">
-        <v>0.704225352112676</v>
+        <v>5.2258064516129</v>
       </c>
       <c r="K19" t="n">
-        <v>0.295774647887324</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="L19" t="n">
-        <v>0.112676056338028</v>
-      </c>
-      <c r="M19"/>
+        <v>0.148148148148148</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B20" t="n">
         <v>42.0420560747664</v>
@@ -1310,22 +1286,21 @@
         <v>0.497674418604651</v>
       </c>
       <c r="I20" t="n">
-        <v>0.0246305418719212</v>
+        <v>11.3883495145631</v>
       </c>
       <c r="J20" t="n">
-        <v>0.58252427184466</v>
+        <v>5.22459893048128</v>
       </c>
       <c r="K20" t="n">
-        <v>0.37378640776699</v>
+        <v>0.208333333333333</v>
       </c>
       <c r="L20" t="n">
-        <v>0.087378640776699</v>
-      </c>
-      <c r="M20"/>
+        <v>0.156976744186047</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B21" t="n">
         <v>41.8551724137931</v>
@@ -1349,22 +1324,21 @@
         <v>0.510344827586207</v>
       </c>
       <c r="I21" t="n">
-        <v>0.041958041958042</v>
+        <v>10.75</v>
       </c>
       <c r="J21" t="n">
-        <v>0.514705882352941</v>
+        <v>4.91240875912409</v>
       </c>
       <c r="K21" t="n">
-        <v>0.279411764705882</v>
+        <v>0.174825174825175</v>
       </c>
       <c r="L21" t="n">
-        <v>0.0661764705882353</v>
-      </c>
-      <c r="M21"/>
+        <v>0.112068965517241</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B22" t="n">
         <v>41.5</v>
@@ -1388,22 +1362,21 @@
         <v>0.513888888888889</v>
       </c>
       <c r="I22" t="n">
-        <v>0.0294117647058824</v>
+        <v>10.3263888888889</v>
       </c>
       <c r="J22" t="n">
-        <v>0.5</v>
+        <v>5.50793650793651</v>
       </c>
       <c r="K22" t="n">
-        <v>0.256944444444444</v>
+        <v>0.0958904109589041</v>
       </c>
       <c r="L22" t="n">
-        <v>0.0694444444444444</v>
-      </c>
-      <c r="M22"/>
+        <v>0.157894736842105</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B23" t="n">
         <v>45.6619718309859</v>
@@ -1427,22 +1400,21 @@
         <v>0.597222222222222</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>12.2537313432836</v>
       </c>
       <c r="J23" t="n">
-        <v>0.701492537313433</v>
+        <v>5.42622950819672</v>
       </c>
       <c r="K23" t="n">
-        <v>0.522388059701492</v>
+        <v>0.277777777777778</v>
       </c>
       <c r="L23" t="n">
-        <v>0.208955223880597</v>
-      </c>
-      <c r="M23"/>
+        <v>0.120689655172414</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B24" t="n">
         <v>45.9583333333333</v>
@@ -1466,22 +1438,21 @@
         <v>0.555555555555556</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>10.6231884057971</v>
       </c>
       <c r="J24" t="n">
-        <v>0.521739130434783</v>
+        <v>4.96363636363636</v>
       </c>
       <c r="K24" t="n">
-        <v>0.304347826086957</v>
+        <v>0.236111111111111</v>
       </c>
       <c r="L24" t="n">
-        <v>0.130434782608696</v>
-      </c>
-      <c r="M24"/>
+        <v>0.0701754385964912</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B25" t="n">
         <v>41.5117370892019</v>
@@ -1505,22 +1476,21 @@
         <v>0.506912442396313</v>
       </c>
       <c r="I25" t="n">
-        <v>0.0338164251207729</v>
+        <v>11.3981042654028</v>
       </c>
       <c r="J25" t="n">
-        <v>0.597156398104265</v>
+        <v>5.39080459770115</v>
       </c>
       <c r="K25" t="n">
-        <v>0.398104265402844</v>
+        <v>0.0604651162790698</v>
       </c>
       <c r="L25" t="n">
-        <v>0.0995260663507109</v>
-      </c>
-      <c r="M25"/>
+        <v>0.241379310344828</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B26" t="n">
         <v>41.875</v>
@@ -1544,22 +1514,21 @@
         <v>0.5</v>
       </c>
       <c r="I26" t="n">
-        <v>0.0144927536231884</v>
+        <v>10.4057971014493</v>
       </c>
       <c r="J26" t="n">
-        <v>0.492753623188406</v>
+        <v>5.50980392156863</v>
       </c>
       <c r="K26" t="n">
-        <v>0.376811594202899</v>
+        <v>0.0972222222222222</v>
       </c>
       <c r="L26" t="n">
-        <v>0.0579710144927536</v>
-      </c>
-      <c r="M26"/>
+        <v>0.466666666666667</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B27" t="n">
         <v>41.0144927536232</v>
@@ -1583,22 +1552,21 @@
         <v>0.528571428571429</v>
       </c>
       <c r="I27" t="n">
-        <v>0.0289855072463768</v>
+        <v>12.2686567164179</v>
       </c>
       <c r="J27" t="n">
-        <v>0.73134328358209</v>
+        <v>5.30909090909091</v>
       </c>
       <c r="K27" t="n">
-        <v>0.492537313432836</v>
+        <v>0.138888888888889</v>
       </c>
       <c r="L27" t="n">
-        <v>0.17910447761194</v>
-      </c>
-      <c r="M27"/>
+        <v>0.232558139534884</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B28" t="n">
         <v>40.4647887323944</v>
@@ -1622,22 +1590,21 @@
         <v>0.458333333333333</v>
       </c>
       <c r="I28" t="n">
-        <v>0.0147058823529412</v>
+        <v>11.7205882352941</v>
       </c>
       <c r="J28" t="n">
-        <v>0.720588235294118</v>
+        <v>5.75862068965517</v>
       </c>
       <c r="K28" t="n">
-        <v>0.367647058823529</v>
+        <v>0.138888888888889</v>
       </c>
       <c r="L28" t="n">
-        <v>0.117647058823529</v>
-      </c>
-      <c r="M28"/>
+        <v>0.172413793103448</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B29" t="n">
         <v>41.6083916083916</v>
@@ -1661,22 +1628,21 @@
         <v>0.4</v>
       </c>
       <c r="I29" t="n">
-        <v>0.0507246376811594</v>
+        <v>11.5174825174825</v>
       </c>
       <c r="J29" t="n">
-        <v>0.65034965034965</v>
+        <v>5.26984126984127</v>
       </c>
       <c r="K29" t="n">
-        <v>0.384615384615385</v>
+        <v>0.158620689655172</v>
       </c>
       <c r="L29" t="n">
-        <v>0.0839160839160839</v>
-      </c>
-      <c r="M29"/>
+        <v>0.151785714285714</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B30" t="n">
         <v>40.2159090909091</v>
@@ -1700,22 +1666,21 @@
         <v>0.5</v>
       </c>
       <c r="I30" t="n">
-        <v>0.0657894736842105</v>
+        <v>9.28888888888889</v>
       </c>
       <c r="J30" t="n">
-        <v>0.355555555555556</v>
+        <v>5.94117647058824</v>
       </c>
       <c r="K30" t="n">
-        <v>0.2</v>
+        <v>0.0666666666666667</v>
       </c>
       <c r="L30" t="n">
-        <v>0.0777777777777778</v>
-      </c>
-      <c r="M30"/>
+        <v>0.230769230769231</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B31" t="n">
         <v>41.7123287671233</v>
@@ -1739,22 +1704,21 @@
         <v>0.493150684931507</v>
       </c>
       <c r="I31" t="n">
-        <v>0.0625</v>
+        <v>8.67123287671233</v>
       </c>
       <c r="J31" t="n">
-        <v>0.301369863013699</v>
+        <v>6.94339622641509</v>
       </c>
       <c r="K31" t="n">
-        <v>0.123287671232877</v>
+        <v>0.0958904109589041</v>
       </c>
       <c r="L31" t="n">
-        <v>0.0273972602739726</v>
-      </c>
-      <c r="M31"/>
+        <v>0.236363636363636</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B32" t="n">
         <v>43.4528301886792</v>
@@ -1778,22 +1742,21 @@
         <v>0.37037037037037</v>
       </c>
       <c r="I32" t="n">
-        <v>0.0416666666666667</v>
+        <v>9.24074074074074</v>
       </c>
       <c r="J32" t="n">
-        <v>0.425925925925926</v>
+        <v>5.325</v>
       </c>
       <c r="K32" t="n">
-        <v>0.240740740740741</v>
+        <v>0.0925925925925926</v>
       </c>
       <c r="L32" t="n">
-        <v>0.0740740740740741</v>
-      </c>
-      <c r="M32"/>
+        <v>0.131578947368421</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B33" t="n">
         <v>39.7361111111111</v>
@@ -1817,22 +1780,21 @@
         <v>0.597222222222222</v>
       </c>
       <c r="I33" t="n">
-        <v>0.112903225806452</v>
+        <v>7.95833333333333</v>
       </c>
       <c r="J33" t="n">
-        <v>0.166666666666667</v>
+        <v>6.36842105263158</v>
       </c>
       <c r="K33" t="n">
-        <v>0.0972222222222222</v>
+        <v>0.138888888888889</v>
       </c>
       <c r="L33" t="n">
-        <v>0.0416666666666667</v>
-      </c>
-      <c r="M33"/>
+        <v>0.169811320754717</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B34" t="n">
         <v>39.4305555555556</v>
@@ -1856,22 +1818,21 @@
         <v>0.388888888888889</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>9.94285714285714</v>
       </c>
       <c r="J34" t="n">
-        <v>0.457142857142857</v>
+        <v>4.65909090909091</v>
       </c>
       <c r="K34" t="n">
-        <v>0.228571428571429</v>
+        <v>0.0416666666666667</v>
       </c>
       <c r="L34" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="M34"/>
+        <v>0.244444444444444</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B35" t="n">
         <v>42.5277777777778</v>
@@ -1895,22 +1856,21 @@
         <v>0.555555555555556</v>
       </c>
       <c r="I35" t="n">
-        <v>0.03125</v>
+        <v>10.5352112676056</v>
       </c>
       <c r="J35" t="n">
-        <v>0.492957746478873</v>
+        <v>5.83333333333333</v>
       </c>
       <c r="K35" t="n">
-        <v>0.253521126760563</v>
+        <v>0.0972222222222222</v>
       </c>
       <c r="L35" t="n">
-        <v>0.126760563380282</v>
-      </c>
-      <c r="M35"/>
+        <v>0.0923076923076923</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B36" t="n">
         <v>42.4305555555556</v>
@@ -1934,22 +1894,21 @@
         <v>0.541666666666667</v>
       </c>
       <c r="I36" t="n">
-        <v>0.0298507462686567</v>
+        <v>10.9154929577465</v>
       </c>
       <c r="J36" t="n">
-        <v>0.507042253521127</v>
+        <v>5.13559322033898</v>
       </c>
       <c r="K36" t="n">
-        <v>0.309859154929577</v>
+        <v>0.180555555555556</v>
       </c>
       <c r="L36" t="n">
-        <v>0.154929577464789</v>
-      </c>
-      <c r="M36"/>
+        <v>0.135593220338983</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B37" t="n">
         <v>41.1527777777778</v>
@@ -1973,22 +1932,21 @@
         <v>0.555555555555556</v>
       </c>
       <c r="I37" t="n">
-        <v>0.0769230769230769</v>
+        <v>10.3888888888889</v>
       </c>
       <c r="J37" t="n">
-        <v>0.472222222222222</v>
+        <v>5.55932203389831</v>
       </c>
       <c r="K37" t="n">
-        <v>0.194444444444444</v>
+        <v>0.263888888888889</v>
       </c>
       <c r="L37" t="n">
-        <v>0.0555555555555556</v>
-      </c>
-      <c r="M37"/>
+        <v>0.178571428571429</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B38" t="n">
         <v>41.9305555555556</v>
@@ -2012,22 +1970,21 @@
         <v>0.527777777777778</v>
       </c>
       <c r="I38" t="n">
-        <v>0.0579710144927536</v>
+        <v>9.65277777777778</v>
       </c>
       <c r="J38" t="n">
-        <v>0.361111111111111</v>
+        <v>5.29411764705882</v>
       </c>
       <c r="K38" t="n">
-        <v>0.208333333333333</v>
+        <v>0.111111111111111</v>
       </c>
       <c r="L38" t="n">
-        <v>0.111111111111111</v>
-      </c>
-      <c r="M38"/>
+        <v>0.12280701754386</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B39" t="n">
         <v>40.4305555555556</v>
@@ -2051,22 +2008,21 @@
         <v>0.472222222222222</v>
       </c>
       <c r="I39" t="n">
-        <v>0.0158730158730159</v>
+        <v>10.5652173913043</v>
       </c>
       <c r="J39" t="n">
-        <v>0.463768115942029</v>
+        <v>5.30645161290323</v>
       </c>
       <c r="K39" t="n">
-        <v>0.27536231884058</v>
+        <v>0.140845070422535</v>
       </c>
       <c r="L39" t="n">
-        <v>0.115942028985507</v>
-      </c>
-      <c r="M39"/>
+        <v>0.160714285714286</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B40" t="n">
         <v>41.9166666666667</v>
@@ -2090,22 +2046,21 @@
         <v>0.583333333333333</v>
       </c>
       <c r="I40" t="n">
-        <v>0.0144927536231884</v>
+        <v>9.88571428571429</v>
       </c>
       <c r="J40" t="n">
-        <v>0.357142857142857</v>
+        <v>5.38235294117647</v>
       </c>
       <c r="K40" t="n">
-        <v>0.2</v>
+        <v>0.208333333333333</v>
       </c>
       <c r="L40" t="n">
-        <v>0.0428571428571429</v>
-      </c>
-      <c r="M40"/>
+        <v>0.1875</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B41" t="n">
         <v>43.9861111111111</v>
@@ -2129,22 +2084,21 @@
         <v>0.430555555555556</v>
       </c>
       <c r="I41" t="n">
-        <v>0.0571428571428571</v>
+        <v>12.8676470588235</v>
       </c>
       <c r="J41" t="n">
-        <v>0.735294117647059</v>
+        <v>4.84615384615385</v>
       </c>
       <c r="K41" t="n">
-        <v>0.455882352941176</v>
+        <v>0.194444444444444</v>
       </c>
       <c r="L41" t="n">
-        <v>0.235294117647059</v>
-      </c>
-      <c r="M41"/>
+        <v>0.0727272727272727</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B42" t="n">
         <v>40.1944444444444</v>
@@ -2168,22 +2122,21 @@
         <v>0.465277777777778</v>
       </c>
       <c r="I42" t="n">
-        <v>0.0510948905109489</v>
+        <v>8.51388888888889</v>
       </c>
       <c r="J42" t="n">
-        <v>0.243055555555556</v>
+        <v>5.16379310344828</v>
       </c>
       <c r="K42" t="n">
-        <v>0.131944444444444</v>
+        <v>0.105633802816901</v>
       </c>
       <c r="L42" t="n">
-        <v>0.0277777777777778</v>
-      </c>
-      <c r="M42"/>
+        <v>0.160714285714286</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B43" t="n">
         <v>41.0416666666667</v>
@@ -2207,22 +2160,21 @@
         <v>0.347222222222222</v>
       </c>
       <c r="I43" t="n">
-        <v>0.0303030303030303</v>
+        <v>10.4084507042254</v>
       </c>
       <c r="J43" t="n">
-        <v>0.408450704225352</v>
+        <v>5.81666666666667</v>
       </c>
       <c r="K43" t="n">
-        <v>0.211267605633803</v>
+        <v>0.169014084507042</v>
       </c>
       <c r="L43" t="n">
-        <v>0.0985915492957746</v>
-      </c>
-      <c r="M43"/>
+        <v>0.203703703703704</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B44" t="n">
         <v>41.6651376146789</v>
@@ -2246,22 +2198,21 @@
         <v>0.488479262672811</v>
       </c>
       <c r="I44" t="n">
-        <v>0.0364583333333333</v>
+        <v>10.0330188679245</v>
       </c>
       <c r="J44" t="n">
-        <v>0.429245283018868</v>
+        <v>5.16292134831461</v>
       </c>
       <c r="K44" t="n">
-        <v>0.240566037735849</v>
+        <v>0.165137614678899</v>
       </c>
       <c r="L44" t="n">
-        <v>0.0754716981132075</v>
-      </c>
-      <c r="M44"/>
+        <v>0.151898734177215</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B45" t="n">
         <v>41.7777777777778</v>
@@ -2285,22 +2236,21 @@
         <v>0.416666666666667</v>
       </c>
       <c r="I45" t="n">
-        <v>0.0434782608695652</v>
+        <v>12.1739130434783</v>
       </c>
       <c r="J45" t="n">
-        <v>0.710144927536232</v>
+        <v>5.4375</v>
       </c>
       <c r="K45" t="n">
-        <v>0.347826086956522</v>
+        <v>0.152777777777778</v>
       </c>
       <c r="L45" t="n">
-        <v>0.159420289855072</v>
-      </c>
-      <c r="M45"/>
+        <v>0.0363636363636364</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B46" t="n">
         <v>42.1369863013699</v>
@@ -2324,22 +2274,21 @@
         <v>0.520547945205479</v>
       </c>
       <c r="I46" t="n">
-        <v>0.109375</v>
+        <v>11.0547945205479</v>
       </c>
       <c r="J46" t="n">
-        <v>0.589041095890411</v>
+        <v>5.57746478873239</v>
       </c>
       <c r="K46" t="n">
-        <v>0.342465753424658</v>
+        <v>0.123287671232877</v>
       </c>
       <c r="L46" t="n">
-        <v>0.136986301369863</v>
-      </c>
-      <c r="M46"/>
+        <v>0.0833333333333333</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B47" t="n">
         <v>43.0416666666667</v>
@@ -2363,22 +2312,21 @@
         <v>0.430555555555556</v>
       </c>
       <c r="I47" t="n">
-        <v>0.0508474576271186</v>
+        <v>10.5714285714286</v>
       </c>
       <c r="J47" t="n">
-        <v>0.528571428571429</v>
+        <v>5.49152542372881</v>
       </c>
       <c r="K47" t="n">
-        <v>0.2</v>
+        <v>0.0833333333333333</v>
       </c>
       <c r="L47" t="n">
-        <v>0.0142857142857143</v>
-      </c>
-      <c r="M47"/>
+        <v>0.169491525423729</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B48" t="n">
         <v>41.3333333333333</v>
@@ -2402,22 +2350,21 @@
         <v>0.625</v>
       </c>
       <c r="I48" t="n">
+        <v>9.65277777777778</v>
+      </c>
+      <c r="J48" t="n">
+        <v>5.859375</v>
+      </c>
+      <c r="K48" t="n">
         <v>0.0277777777777778</v>
       </c>
-      <c r="J48" t="n">
-        <v>0.388888888888889</v>
-      </c>
-      <c r="K48" t="n">
-        <v>0.25</v>
-      </c>
       <c r="L48" t="n">
-        <v>0.0555555555555556</v>
-      </c>
-      <c r="M48"/>
+        <v>0.15</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B49" t="n">
         <v>42.397212543554</v>
@@ -2441,22 +2388,21 @@
         <v>0.522491349480969</v>
       </c>
       <c r="I49" t="n">
-        <v>0.0255474452554745</v>
+        <v>10.8140350877193</v>
       </c>
       <c r="J49" t="n">
-        <v>0.519298245614035</v>
+        <v>5.30555555555556</v>
       </c>
       <c r="K49" t="n">
-        <v>0.301754385964912</v>
+        <v>0.118466898954704</v>
       </c>
       <c r="L49" t="n">
-        <v>0.101754385964912</v>
-      </c>
-      <c r="M49"/>
+        <v>0.146788990825688</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B50" t="n">
         <v>44.1</v>
@@ -2480,22 +2426,21 @@
         <v>0.436619718309859</v>
       </c>
       <c r="I50" t="n">
-        <v>0.0153846153846154</v>
+        <v>9.49295774647887</v>
       </c>
       <c r="J50" t="n">
-        <v>0.309859154929577</v>
+        <v>5.13559322033898</v>
       </c>
       <c r="K50" t="n">
-        <v>0.169014084507042</v>
+        <v>0.0704225352112676</v>
       </c>
       <c r="L50" t="n">
-        <v>0.0422535211267606</v>
-      </c>
-      <c r="M50"/>
+        <v>0.259259259259259</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B51" t="n">
         <v>41.5103448275862</v>
@@ -2519,22 +2464,21 @@
         <v>0.631944444444444</v>
       </c>
       <c r="I51" t="n">
-        <v>0.1</v>
+        <v>9.53103448275862</v>
       </c>
       <c r="J51" t="n">
-        <v>0.358620689655172</v>
+        <v>5.5045045045045</v>
       </c>
       <c r="K51" t="n">
-        <v>0.151724137931034</v>
+        <v>0.110344827586207</v>
       </c>
       <c r="L51" t="n">
-        <v>0.0275862068965517</v>
-      </c>
-      <c r="M51"/>
+        <v>0.104761904761905</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B52" t="n">
         <v>40.5333333333333</v>
@@ -2558,22 +2502,21 @@
         <v>0.546666666666667</v>
       </c>
       <c r="I52" t="n">
-        <v>0.0166666666666667</v>
+        <v>8.30666666666667</v>
       </c>
       <c r="J52" t="n">
-        <v>0.306666666666667</v>
+        <v>6.14285714285714</v>
       </c>
       <c r="K52" t="n">
-        <v>0.0666666666666667</v>
+        <v>0.0945945945945946</v>
       </c>
       <c r="L52" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="M52"/>
+        <v>0.290909090909091</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B53" t="n">
         <v>41.1388888888889</v>
@@ -2597,22 +2540,21 @@
         <v>0.534722222222222</v>
       </c>
       <c r="I53" t="n">
-        <v>0.0508474576271186</v>
+        <v>7.89583333333333</v>
       </c>
       <c r="J53" t="n">
-        <v>0.270833333333333</v>
+        <v>6.58914728682171</v>
       </c>
       <c r="K53" t="n">
-        <v>0.0694444444444444</v>
+        <v>0.0625</v>
       </c>
       <c r="L53" t="n">
-        <v>0</v>
-      </c>
-      <c r="M53"/>
+        <v>0.194174757281553</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B54" t="n">
         <v>41.656462585034</v>
@@ -2636,22 +2578,21 @@
         <v>0.496598639455782</v>
       </c>
       <c r="I54" t="n">
-        <v>0.0252707581227437</v>
+        <v>9.92631578947368</v>
       </c>
       <c r="J54" t="n">
-        <v>0.435087719298246</v>
+        <v>5.97881355932203</v>
       </c>
       <c r="K54" t="n">
-        <v>0.217543859649123</v>
+        <v>0.126279863481229</v>
       </c>
       <c r="L54" t="n">
-        <v>0.056140350877193</v>
-      </c>
-      <c r="M54"/>
+        <v>0.152</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B55" t="n">
         <v>39.9014084507042</v>
@@ -2675,18 +2616,17 @@
         <v>0.520547945205479</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
+        <v>10.7571428571429</v>
       </c>
       <c r="J55" t="n">
-        <v>0.542857142857143</v>
+        <v>6.64516129032258</v>
       </c>
       <c r="K55" t="n">
-        <v>0.185714285714286</v>
+        <v>0.0684931506849315</v>
       </c>
       <c r="L55" t="n">
-        <v>0.0571428571428571</v>
-      </c>
-      <c r="M55"/>
+        <v>0.238095238095238</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>